<commit_message>
feat: branded HTML report + correct SP mapping + Drive upload
</commit_message>
<xml_diff>
--- a/MCL_Portfolio_LIVE.xlsx
+++ b/MCL_Portfolio_LIVE.xlsx
@@ -9,12 +9,11 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Branch Arrears" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Loan Products" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Loan Category" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Loan Category" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Category by Branch" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Active Loans" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Total Balance" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Principal Balance" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Portfolio Arrears" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00&quot;%&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,6 +93,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C53030"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="12">
@@ -249,9 +253,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -264,6 +265,7 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
@@ -632,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -653,7 +655,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As at Date: 2026-06-21    |    All Branches    |    Database: mwananchidy365    |    Generated: 21 Jun 2026 16:57</t>
+          <t>As at Date: 2026-06-21    |    All Branches    |    Database: mwananchidy365    |    Generated: 21 Jun 2026 18:36</t>
         </is>
       </c>
     </row>
@@ -722,39 +724,35 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>PORTFOLIO AT RISK</t>
+          <t>PORTFOLIO AT RISK (PAR)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>2,520,942,495.52</t>
-        </is>
+      <c r="A9" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>11501</v>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>51.01 %</t>
-        </is>
+        <v>2340</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10" ht="12" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>KES</t>
+          <t>KES — Watch 1+ only</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>accounts overdue</t>
+          <t>accounts — Watch 1+ only</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>PAR %</t>
+          <t>PAR % (excl. Performing)</t>
         </is>
       </c>
     </row>
@@ -795,41 +793,41 @@
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Portfolio in arrears by branch — loan count, arrears amount, balance, PAR%</t>
+          <t>Branch-level arrears, outstanding balance and PAR%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="inlineStr">
         <is>
-          <t>Loan Products</t>
+          <t>Loan Category</t>
         </is>
       </c>
       <c r="B16" s="16" t="inlineStr">
         <is>
-          <t>sp_PortfolioByLoanProduct</t>
+          <t>sp_PortfolioByLoanCategory</t>
         </is>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>Portfolio breakdown by loan product type</t>
+          <t>Watch 1+ arrears section + Performing section (separated). Arrears KPIs derived from this SP.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Loan Category</t>
+          <t>Category by Branch</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>sp_PortfolioByLoanCategory</t>
+          <t>sp_PortfolioArrearsByBranchArrears</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Portfolio by credit classification (Performing, Watch, Substandard, Doubtful, Loss)</t>
+          <t>Loan category arrears breakdown per branch (Watch 1+ only, Performing excluded)</t>
         </is>
       </c>
     </row>
@@ -846,7 +844,7 @@
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>Total count of active loans</t>
+          <t>Total count of active loans in the portfolio</t>
         </is>
       </c>
     </row>
@@ -881,23 +879,6 @@
       <c r="C20" s="16" t="inlineStr">
         <is>
           <t>Principal outstanding balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Portfolio Arrears</t>
-        </is>
-      </c>
-      <c r="B21" s="15" t="inlineStr">
-        <is>
-          <t>sp_Portfoliainarrears</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
-        <is>
-          <t>Overall portfolio in arrears — total amount, count, PAR%</t>
         </is>
       </c>
     </row>
@@ -957,7 +938,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Branch-level arrears, loan balance and PAR percentage  |  SP: sp_PortfolioInArrearsByBranch  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 16:57</t>
+          <t>Branch-level arrears, loan balance and PAR % (Watch 1+ only)  |  SP: sp_PortfolioInArrearsByBranch  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:36</t>
         </is>
       </c>
     </row>
@@ -1035,21 +1016,21 @@
         </is>
       </c>
       <c r="C6" s="22" t="n">
-        <v>1142</v>
+        <v>1146</v>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>691,827,683.17</t>
+          <t>696,852,812.30</t>
         </is>
       </c>
       <c r="E6" s="23" t="inlineStr">
         <is>
-          <t>958,347,978.22</t>
+          <t>966,037,478.22</t>
         </is>
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
-          <t>72.19 %</t>
+          <t>72.14 %</t>
         </is>
       </c>
     </row>
@@ -1065,21 +1046,21 @@
         </is>
       </c>
       <c r="C7" s="19" t="n">
-        <v>1271</v>
+        <v>1279</v>
       </c>
       <c r="D7" s="20" t="inlineStr">
         <is>
-          <t>448,653,730.40</t>
+          <t>448,789,785.49</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
-          <t>752,393,568.72</t>
+          <t>754,123,127.59</t>
         </is>
       </c>
       <c r="F7" s="21" t="inlineStr">
         <is>
-          <t>59.63 %</t>
+          <t>59.51 %</t>
         </is>
       </c>
     </row>
@@ -1095,21 +1076,21 @@
         </is>
       </c>
       <c r="C8" s="22" t="n">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="D8" s="23" t="inlineStr">
         <is>
-          <t>163,253,624.82</t>
+          <t>163,407,374.82</t>
         </is>
       </c>
       <c r="E8" s="23" t="inlineStr">
         <is>
-          <t>289,949,861.55</t>
+          <t>290,874,612.55</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>56.30 %</t>
+          <t>56.18 %</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1106,7 @@
         </is>
       </c>
       <c r="C9" s="19" t="n">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="D9" s="20" t="inlineStr">
         <is>
@@ -1134,7 +1115,7 @@
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>286,927,714.40</t>
+          <t>286,953,814.40</t>
         </is>
       </c>
       <c r="F9" s="21" t="inlineStr">
@@ -1155,21 +1136,21 @@
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>620,530,442.57</t>
+          <t>620,547,382.57</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>617,139,245.11</t>
+          <t>617,305,515.11</t>
         </is>
       </c>
       <c r="F10" s="24" t="inlineStr">
         <is>
-          <t>100.55 %</t>
+          <t>100.53 %</t>
         </is>
       </c>
     </row>
@@ -1185,21 +1166,21 @@
         </is>
       </c>
       <c r="C11" s="19" t="n">
-        <v>899</v>
+        <v>902</v>
       </c>
       <c r="D11" s="20" t="inlineStr">
         <is>
-          <t>159,928,685.36</t>
+          <t>159,985,146.57</t>
         </is>
       </c>
       <c r="E11" s="20" t="inlineStr">
         <is>
-          <t>269,325,671.26</t>
+          <t>269,812,217.35</t>
         </is>
       </c>
       <c r="F11" s="21" t="inlineStr">
         <is>
-          <t>59.38 %</t>
+          <t>59.29 %</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1256,7 @@
         </is>
       </c>
       <c r="C14" s="22" t="n">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
@@ -1284,12 +1265,12 @@
       </c>
       <c r="E14" s="23" t="inlineStr">
         <is>
-          <t>161,176,998.65</t>
+          <t>161,276,998.65</t>
         </is>
       </c>
       <c r="F14" s="24" t="inlineStr">
         <is>
-          <t>14.44 %</t>
+          <t>14.43 %</t>
         </is>
       </c>
     </row>
@@ -1305,21 +1286,21 @@
         </is>
       </c>
       <c r="C15" s="19" t="n">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="D15" s="20" t="inlineStr">
         <is>
-          <t>19,206,205.79</t>
+          <t>19,207,453.61</t>
         </is>
       </c>
       <c r="E15" s="20" t="inlineStr">
         <is>
-          <t>144,201,941.54</t>
+          <t>144,290,306.44</t>
         </is>
       </c>
       <c r="F15" s="21" t="inlineStr">
         <is>
-          <t>13.32 %</t>
+          <t>13.31 %</t>
         </is>
       </c>
     </row>
@@ -1335,21 +1316,21 @@
         </is>
       </c>
       <c r="C16" s="22" t="n">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>7,750,046.47</t>
+          <t>7,756,260.47</t>
         </is>
       </c>
       <c r="E16" s="23" t="inlineStr">
         <is>
-          <t>84,992,442.33</t>
+          <t>85,145,551.33</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>9.12 %</t>
+          <t>9.11 %</t>
         </is>
       </c>
     </row>
@@ -1453,21 +1434,21 @@
         </is>
       </c>
       <c r="C20" s="22" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D20" s="23" t="inlineStr">
         <is>
-          <t>3,209,386.56</t>
+          <t>3,241,664.36</t>
         </is>
       </c>
       <c r="E20" s="23" t="inlineStr">
         <is>
-          <t>32,726,644.80</t>
+          <t>33,520,591.00</t>
         </is>
       </c>
       <c r="F20" s="24" t="inlineStr">
         <is>
-          <t>9.81 %</t>
+          <t>9.67 %</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1490,7 @@
       </c>
       <c r="B22" s="26" t="inlineStr"/>
       <c r="C22" s="27" t="n">
-        <v>11501</v>
+        <v>11530</v>
       </c>
       <c r="D22" s="26" t="inlineStr"/>
       <c r="E22" s="26" t="inlineStr"/>
@@ -1525,829 +1506,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Z35"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>MWANANCHI CREDIT LTD — PORTFOLIO BY LOAN PRODUCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
-        <is>
-          <t>Arrears and balance breakdown by loan product type  |  SP: sp_PortfolioByLoanProduct  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 16:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>LoanProductType</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>LoanCount</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>TotalAmountInArrears</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>LoanBalance</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="inlineStr">
-        <is>
-          <t>PercentageInArrears</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
-        <is>
-          <t>Assest Finance</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="n">
-        <v>8</v>
-      </c>
-      <c r="C5" s="20" t="inlineStr">
-        <is>
-          <t>9,851,249.66</t>
-        </is>
-      </c>
-      <c r="D5" s="20" t="inlineStr">
-        <is>
-          <t>4,353,067.69</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
-          <t>226.31 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>Asset Finance</t>
-        </is>
-      </c>
-      <c r="B6" s="22" t="n">
-        <v>20</v>
-      </c>
-      <c r="C6" s="23" t="inlineStr">
-        <is>
-          <t>626,721.83</t>
-        </is>
-      </c>
-      <c r="D6" s="23" t="inlineStr">
-        <is>
-          <t>26,661,076.67</t>
-        </is>
-      </c>
-      <c r="E6" s="24" t="inlineStr">
-        <is>
-          <t>2.35 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>Boda Boda Financing</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="n">
-        <v>62</v>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>14,424,902.64</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>6,264,849.06</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>230.25 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>Checkoff</t>
-        </is>
-      </c>
-      <c r="B8" s="22" t="n">
-        <v>9108</v>
-      </c>
-      <c r="C8" s="23" t="inlineStr">
-        <is>
-          <t>194,558,671.15</t>
-        </is>
-      </c>
-      <c r="D8" s="23" t="inlineStr">
-        <is>
-          <t>2,671,331,578.02</t>
-        </is>
-      </c>
-      <c r="E8" s="24" t="inlineStr">
-        <is>
-          <t>7.28 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>Cheque Discounting</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="C9" s="20" t="inlineStr">
-        <is>
-          <t>7,969,270.70</t>
-        </is>
-      </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>13,369,539.70</t>
-        </is>
-      </c>
-      <c r="E9" s="21" t="inlineStr">
-        <is>
-          <t>59.61 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>CHEQUE DISCOUNTING</t>
-        </is>
-      </c>
-      <c r="B10" s="22" t="n">
-        <v>9</v>
-      </c>
-      <c r="C10" s="23" t="inlineStr">
-        <is>
-          <t>1,359,897.01</t>
-        </is>
-      </c>
-      <c r="D10" s="23" t="inlineStr">
-        <is>
-          <t>1,286,370.18</t>
-        </is>
-      </c>
-      <c r="E10" s="24" t="inlineStr">
-        <is>
-          <t>105.72 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="15" t="inlineStr">
-        <is>
-          <t>Import Duty</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>2,971,170.73</t>
-        </is>
-      </c>
-      <c r="D11" s="20" t="inlineStr">
-        <is>
-          <t>1,352,839.00</t>
-        </is>
-      </c>
-      <c r="E11" s="21" t="inlineStr">
-        <is>
-          <t>219.62 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="16" t="inlineStr">
-        <is>
-          <t>Import Duty Finance</t>
-        </is>
-      </c>
-      <c r="B12" s="22" t="n">
-        <v>3</v>
-      </c>
-      <c r="C12" s="23" t="inlineStr">
-        <is>
-          <t>10,010,553.95</t>
-        </is>
-      </c>
-      <c r="D12" s="23" t="inlineStr">
-        <is>
-          <t>5,208,760.00</t>
-        </is>
-      </c>
-      <c r="E12" s="24" t="inlineStr">
-        <is>
-          <t>192.19 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Insurance Premium Finance </t>
-        </is>
-      </c>
-      <c r="B13" s="19" t="n">
-        <v>91</v>
-      </c>
-      <c r="C13" s="20" t="inlineStr">
-        <is>
-          <t>2,585,579.43</t>
-        </is>
-      </c>
-      <c r="D13" s="20" t="inlineStr">
-        <is>
-          <t>6,705,894.69</t>
-        </is>
-      </c>
-      <c r="E13" s="21" t="inlineStr">
-        <is>
-          <t>38.56 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="16" t="inlineStr">
-        <is>
-          <t>LOG BOOK LOAN</t>
-        </is>
-      </c>
-      <c r="B14" s="22" t="n">
-        <v>9</v>
-      </c>
-      <c r="C14" s="23" t="inlineStr">
-        <is>
-          <t>8,604,544.17</t>
-        </is>
-      </c>
-      <c r="D14" s="23" t="inlineStr">
-        <is>
-          <t>3,192,351.43</t>
-        </is>
-      </c>
-      <c r="E14" s="24" t="inlineStr">
-        <is>
-          <t>269.54 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>Logbook</t>
-        </is>
-      </c>
-      <c r="B15" s="19" t="n">
-        <v>994</v>
-      </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>534,636,849.11</t>
-        </is>
-      </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>620,309,254.74</t>
-        </is>
-      </c>
-      <c r="E15" s="21" t="inlineStr">
-        <is>
-          <t>86.19 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>LOGBOOK</t>
-        </is>
-      </c>
-      <c r="B16" s="22" t="n">
-        <v>310</v>
-      </c>
-      <c r="C16" s="23" t="inlineStr">
-        <is>
-          <t>539,601,332.65</t>
-        </is>
-      </c>
-      <c r="D16" s="23" t="inlineStr">
-        <is>
-          <t>154,046,807.60</t>
-        </is>
-      </c>
-      <c r="E16" s="24" t="inlineStr">
-        <is>
-          <t>350.28 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>LOGBOOK &amp; TD</t>
-        </is>
-      </c>
-      <c r="B17" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C17" s="20" t="inlineStr">
-        <is>
-          <t>69,581,843.82</t>
-        </is>
-      </c>
-      <c r="D17" s="20" t="inlineStr">
-        <is>
-          <t>24,396,649.73</t>
-        </is>
-      </c>
-      <c r="E17" s="21" t="inlineStr">
-        <is>
-          <t>285.21 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="16" t="inlineStr">
-        <is>
-          <t>Logbook Capitalized</t>
-        </is>
-      </c>
-      <c r="B18" s="22" t="n">
-        <v>4</v>
-      </c>
-      <c r="C18" s="23" t="inlineStr">
-        <is>
-          <t>3,096,849.27</t>
-        </is>
-      </c>
-      <c r="D18" s="23" t="inlineStr">
-        <is>
-          <t>5,231,325.31</t>
-        </is>
-      </c>
-      <c r="E18" s="24" t="inlineStr">
-        <is>
-          <t>59.20 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>Mobile Loan - Logbook</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="n">
-        <v>135</v>
-      </c>
-      <c r="C19" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="20" t="inlineStr">
-        <is>
-          <t>12,101,945.00</t>
-        </is>
-      </c>
-      <c r="E19" s="21" t="inlineStr">
-        <is>
-          <t>0.00 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>Mobile Loan - Title Deed</t>
-        </is>
-      </c>
-      <c r="B20" s="22" t="n">
-        <v>2</v>
-      </c>
-      <c r="C20" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="23" t="inlineStr">
-        <is>
-          <t>354,400.00</t>
-        </is>
-      </c>
-      <c r="E20" s="24" t="inlineStr">
-        <is>
-          <t>0.00 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Salary Advance</t>
-        </is>
-      </c>
-      <c r="B21" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C21" s="20" t="inlineStr">
-        <is>
-          <t>349,933.07</t>
-        </is>
-      </c>
-      <c r="D21" s="20" t="inlineStr">
-        <is>
-          <t>146,598.00</t>
-        </is>
-      </c>
-      <c r="E21" s="21" t="inlineStr">
-        <is>
-          <t>238.70 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1">
-      <c r="A22" s="16" t="inlineStr">
-        <is>
-          <t>Staff Loan</t>
-        </is>
-      </c>
-      <c r="B22" s="22" t="n">
-        <v>19</v>
-      </c>
-      <c r="C22" s="23" t="inlineStr">
-        <is>
-          <t>37,353.00</t>
-        </is>
-      </c>
-      <c r="D22" s="23" t="inlineStr">
-        <is>
-          <t>2,411,778.74</t>
-        </is>
-      </c>
-      <c r="E22" s="24" t="inlineStr">
-        <is>
-          <t>1.55 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
-        <is>
-          <t>STAFF LOAN</t>
-        </is>
-      </c>
-      <c r="B23" s="19" t="n">
-        <v>24</v>
-      </c>
-      <c r="C23" s="20" t="inlineStr">
-        <is>
-          <t>1,273,937.99</t>
-        </is>
-      </c>
-      <c r="D23" s="20" t="inlineStr">
-        <is>
-          <t>1,133,599.69</t>
-        </is>
-      </c>
-      <c r="E23" s="21" t="inlineStr">
-        <is>
-          <t>112.38 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>Staff Salary Advance</t>
-        </is>
-      </c>
-      <c r="B24" s="22" t="n">
-        <v>20</v>
-      </c>
-      <c r="C24" s="23" t="inlineStr">
-        <is>
-          <t>998,799.38</t>
-        </is>
-      </c>
-      <c r="D24" s="23" t="inlineStr">
-        <is>
-          <t>1,318,657.35</t>
-        </is>
-      </c>
-      <c r="E24" s="24" t="inlineStr">
-        <is>
-          <t>75.74 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="15" t="inlineStr">
-        <is>
-          <t>Staff Salary Loan</t>
-        </is>
-      </c>
-      <c r="B25" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="20" t="inlineStr">
-        <is>
-          <t>8,850.00</t>
-        </is>
-      </c>
-      <c r="D25" s="20" t="inlineStr">
-        <is>
-          <t>42,300.00</t>
-        </is>
-      </c>
-      <c r="E25" s="21" t="inlineStr">
-        <is>
-          <t>20.92 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>Title Deed</t>
-        </is>
-      </c>
-      <c r="B26" s="22" t="n">
-        <v>154</v>
-      </c>
-      <c r="C26" s="23" t="inlineStr">
-        <is>
-          <t>771,019,866.11</t>
-        </is>
-      </c>
-      <c r="D26" s="23" t="inlineStr">
-        <is>
-          <t>813,244,057.83</t>
-        </is>
-      </c>
-      <c r="E26" s="24" t="inlineStr">
-        <is>
-          <t>94.81 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="15" t="inlineStr">
-        <is>
-          <t>TITLE DEED</t>
-        </is>
-      </c>
-      <c r="B27" s="19" t="n">
-        <v>20</v>
-      </c>
-      <c r="C27" s="20" t="inlineStr">
-        <is>
-          <t>140,279,969.82</t>
-        </is>
-      </c>
-      <c r="D27" s="20" t="inlineStr">
-        <is>
-          <t>30,365,229.74</t>
-        </is>
-      </c>
-      <c r="E27" s="21" t="inlineStr">
-        <is>
-          <t>461.98 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Trade Finance</t>
-        </is>
-      </c>
-      <c r="B28" s="22" t="n">
-        <v>7</v>
-      </c>
-      <c r="C28" s="23" t="inlineStr">
-        <is>
-          <t>14,189,099.60</t>
-        </is>
-      </c>
-      <c r="D28" s="23" t="inlineStr">
-        <is>
-          <t>166,667,598.90</t>
-        </is>
-      </c>
-      <c r="E28" s="24" t="inlineStr">
-        <is>
-          <t>8.51 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="15" t="inlineStr">
-        <is>
-          <t>Unsecured</t>
-        </is>
-      </c>
-      <c r="B29" s="19" t="n">
-        <v>75</v>
-      </c>
-      <c r="C29" s="20" t="inlineStr">
-        <is>
-          <t>64,895,361.29</t>
-        </is>
-      </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>299,672,578.75</t>
-        </is>
-      </c>
-      <c r="E29" s="21" t="inlineStr">
-        <is>
-          <t>21.66 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>UNSECURED</t>
-        </is>
-      </c>
-      <c r="B30" s="22" t="n">
-        <v>280</v>
-      </c>
-      <c r="C30" s="23" t="inlineStr">
-        <is>
-          <t>71,183,862.85</t>
-        </is>
-      </c>
-      <c r="D30" s="23" t="inlineStr">
-        <is>
-          <t>28,625,081.24</t>
-        </is>
-      </c>
-      <c r="E30" s="24" t="inlineStr">
-        <is>
-          <t>248.68 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="15" t="inlineStr">
-        <is>
-          <t>Weekend</t>
-        </is>
-      </c>
-      <c r="B31" s="19" t="n">
-        <v>106</v>
-      </c>
-      <c r="C31" s="20" t="inlineStr">
-        <is>
-          <t>45,862,317.21</t>
-        </is>
-      </c>
-      <c r="D31" s="20" t="inlineStr">
-        <is>
-          <t>37,670,303.26</t>
-        </is>
-      </c>
-      <c r="E31" s="21" t="inlineStr">
-        <is>
-          <t>121.75 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
-        <is>
-          <t>WEEKEND</t>
-        </is>
-      </c>
-      <c r="B32" s="22" t="n">
-        <v>5</v>
-      </c>
-      <c r="C32" s="23" t="inlineStr">
-        <is>
-          <t>1,801,094.20</t>
-        </is>
-      </c>
-      <c r="D32" s="23" t="inlineStr">
-        <is>
-          <t>749,053.88</t>
-        </is>
-      </c>
-      <c r="E32" s="24" t="inlineStr">
-        <is>
-          <t>240.45 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="15" t="inlineStr">
-        <is>
-          <t>Weekend Loan</t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" s="20" t="inlineStr">
-        <is>
-          <t>4,093.54</t>
-        </is>
-      </c>
-      <c r="D33" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="21" t="inlineStr">
-        <is>
-          <t>0.00 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>WEEKEND LOAN</t>
-        </is>
-      </c>
-      <c r="B34" s="22" t="n">
-        <v>18</v>
-      </c>
-      <c r="C34" s="23" t="inlineStr">
-        <is>
-          <t>9,158,521.34</t>
-        </is>
-      </c>
-      <c r="D34" s="23" t="inlineStr">
-        <is>
-          <t>3,582,592.13</t>
-        </is>
-      </c>
-      <c r="E34" s="24" t="inlineStr">
-        <is>
-          <t>255.64 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="26" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B35" s="27" t="n">
-        <v>11501</v>
-      </c>
-      <c r="C35" s="26" t="inlineStr"/>
-      <c r="D35" s="26" t="inlineStr"/>
-      <c r="E35" s="26" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="A2:Z2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2373,12 +1531,12 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Credit classification breakdown  |  sp_PortfolioByLoanCategory  |  As at: 2026-06-21  |  21 Jun 2026 16:57</t>
+          <t>Credit classification breakdown  |  sp_PortfolioByLoanCategory  |  As at: 2026-06-21  |  21 Jun 2026 18:36</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>ARREARS CATEGORIES  —  Watch 1 / Watch 2 / Substandard / Doubtful / Loss</t>
         </is>
@@ -2418,21 +1576,21 @@
         </is>
       </c>
       <c r="B6" s="19" t="n">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>4,199,613.15</t>
+          <t>4,431,869.07</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
-          <t>86,784,307.41</t>
-        </is>
-      </c>
-      <c r="E6" s="30" t="inlineStr">
-        <is>
-          <t>4.84 %</t>
+          <t>89,296,254.22</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
+        <is>
+          <t>4.96 %</t>
         </is>
       </c>
     </row>
@@ -2455,7 +1613,7 @@
           <t>59,351,538.51</t>
         </is>
       </c>
-      <c r="E7" s="31" t="inlineStr">
+      <c r="E7" s="30" t="inlineStr">
         <is>
           <t>3.67 %</t>
         </is>
@@ -2480,7 +1638,7 @@
           <t>26,292,071.83</t>
         </is>
       </c>
-      <c r="E8" s="30" t="inlineStr">
+      <c r="E8" s="29" t="inlineStr">
         <is>
           <t>12.08 %</t>
         </is>
@@ -2505,7 +1663,7 @@
           <t>14,478,940.77</t>
         </is>
       </c>
-      <c r="E9" s="31" t="inlineStr">
+      <c r="E9" s="30" t="inlineStr">
         <is>
           <t>11.01 %</t>
         </is>
@@ -2518,21 +1676,21 @@
         </is>
       </c>
       <c r="B10" s="19" t="n">
-        <v>2032</v>
+        <v>2035</v>
       </c>
       <c r="C10" s="20" t="inlineStr">
         <is>
-          <t>2,507,980,238.98</t>
+          <t>2,513,176,058.11</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
-          <t>1,412,816,523.64</t>
-        </is>
-      </c>
-      <c r="E10" s="30" t="inlineStr">
-        <is>
-          <t>177.52 %</t>
+          <t>1,417,886,028.64</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="inlineStr">
+        <is>
+          <t>177.25 %</t>
         </is>
       </c>
     </row>
@@ -2543,14 +1701,14 @@
         </is>
       </c>
       <c r="B11" s="27" t="n">
-        <v>2327</v>
+        <v>2340</v>
       </c>
       <c r="C11" s="26" t="inlineStr"/>
       <c r="D11" s="26" t="inlineStr"/>
       <c r="E11" s="26" t="inlineStr"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>PERFORMING — CURRENT LOANS (NOT IN ARREARS)</t>
         </is>
@@ -2590,7 +1748,7 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>9174</v>
+        <v>9190</v>
       </c>
       <c r="C15" s="20" t="inlineStr">
         <is>
@@ -2599,10 +1757,10 @@
       </c>
       <c r="D15" s="20" t="inlineStr">
         <is>
-          <t>3,342,072,756.17</t>
-        </is>
-      </c>
-      <c r="E15" s="30" t="inlineStr">
+          <t>3,346,649,450.42</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="inlineStr">
         <is>
           <t>0.05 %</t>
         </is>
@@ -2615,7 +1773,7 @@
         </is>
       </c>
       <c r="B16" s="27" t="n">
-        <v>9174</v>
+        <v>9190</v>
       </c>
       <c r="C16" s="26" t="inlineStr"/>
       <c r="D16" s="26" t="inlineStr"/>
@@ -2626,6 +1784,45 @@
     <mergeCell ref="A1:Z1"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A2:Z2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>MWANANCHI CREDIT LTD — LOAN CATEGORIES BY BRANCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
+      <c r="A2" s="18" t="inlineStr">
+        <is>
+          <t>Arrears breakdown by loan category per branch — Watch 1+ (Performing excluded)  |  SP: sp_PortfolioArrearsByBranchArrears  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>ERROR connecting to sp_PortfolioArrearsByBranchArrears: (2812, b"Could not find stored procedure 'sp_PortfolioArrearsByBranchArrears'.DB-Lib error message 20018, severity 16:\nGeneral SQL Server error: Check messages from the SQL Server\n")</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:Z1"/>
     <mergeCell ref="A2:Z2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2654,7 +1851,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Total number of active loans in the portfolio  |  SP: sp_ActiveLoanCount  |  As at: None  |  Generated: 21 Jun 2026 16:57</t>
+          <t>Total number of active loans in the portfolio  |  SP: sp_ActiveLoanCount  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:37</t>
         </is>
       </c>
     </row>
@@ -2708,7 +1905,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Principal outstanding balance across all active loans  |  SP: sp_TotalLoanBalance  |  As at: None  |  Generated: 21 Jun 2026 16:57</t>
+          <t>Principal outstanding balance across all active loans  |  SP: sp_TotalLoanBalance  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:37</t>
         </is>
       </c>
     </row>
@@ -2762,7 +1959,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Principal outstanding balance  |  SP: sp_LoanPrincipalBalance  |  As at: None  |  Generated: 21 Jun 2026 16:57</t>
+          <t>Principal outstanding balance  |  SP: sp_LoanPrincipalBalance  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:37</t>
         </is>
       </c>
     </row>
@@ -2784,96 +1981,6 @@
           <t>TOTAL</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="A2:Z2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:Z6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>MWANANCHI CREDIT LTD — PORTFOLIO IN ARREARS — OVERALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
-        <is>
-          <t>Total arrears, loan count in arrears, PAR percentage  |  SP: sp_Portfoliainarrears  |  As at: None  |  Generated: 21 Jun 2026 16:57</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
-        <is>
-          <t>LoanCount</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>TotalAmountInArrears</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
-        <is>
-          <t>LoanBalance</t>
-        </is>
-      </c>
-      <c r="D4" s="14" t="inlineStr">
-        <is>
-          <t>PercentageInArrears</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" s="25" t="n">
-        <v>11501</v>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>2,520,942,495.52</t>
-        </is>
-      </c>
-      <c r="C5" s="20" t="inlineStr">
-        <is>
-          <t>4,941,796,138.33</t>
-        </is>
-      </c>
-      <c r="D5" s="15" t="inlineStr">
-        <is>
-          <t>51.01 %</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B6" s="26" t="inlineStr"/>
-      <c r="C6" s="26" t="inlineStr"/>
-      <c r="D6" s="26" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
fix: auto-detect file:// vs Flask, set API_BASE accordingly
</commit_message>
<xml_diff>
--- a/MCL_Portfolio_LIVE.xlsx
+++ b/MCL_Portfolio_LIVE.xlsx
@@ -655,7 +655,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>As at Date: 2026-06-21    |    All Branches    |    Database: mwananchidy365    |    Generated: 21 Jun 2026 18:36</t>
+          <t>As at Date: 2026-06-21    |    All Branches    |    Database: mwananchidy365    |    Generated: 21 Jun 2026 18:47</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Branch-level arrears, loan balance and PAR % (Watch 1+ only)  |  SP: sp_PortfolioInArrearsByBranch  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:36</t>
+          <t>Branch-level arrears, loan balance and PAR % (Watch 1+ only)  |  SP: sp_PortfolioInArrearsByBranch  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:47</t>
         </is>
       </c>
     </row>
@@ -1531,7 +1531,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Credit classification breakdown  |  sp_PortfolioByLoanCategory  |  As at: 2026-06-21  |  21 Jun 2026 18:36</t>
+          <t>Credit classification breakdown  |  sp_PortfolioByLoanCategory  |  As at: 2026-06-21  |  21 Jun 2026 18:47</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Arrears breakdown by loan category per branch — Watch 1+ (Performing excluded)  |  SP: sp_PortfolioArrearsByBranchArrears  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:36</t>
+          <t>Arrears breakdown by loan category per branch — Watch 1+ (Performing excluded)  |  SP: sp_PortfolioArrearsByBranchArrears  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:47</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Total number of active loans in the portfolio  |  SP: sp_ActiveLoanCount  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:37</t>
+          <t>Total number of active loans in the portfolio  |  SP: sp_ActiveLoanCount  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:47</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Principal outstanding balance across all active loans  |  SP: sp_TotalLoanBalance  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:37</t>
+          <t>Principal outstanding balance across all active loans  |  SP: sp_TotalLoanBalance  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:47</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1959,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="18" t="inlineStr">
         <is>
-          <t>Principal outstanding balance  |  SP: sp_LoanPrincipalBalance  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:37</t>
+          <t>Principal outstanding balance  |  SP: sp_LoanPrincipalBalance  |  As at: 2026-06-21  |  Generated: 21 Jun 2026 18:47</t>
         </is>
       </c>
     </row>

</xml_diff>